<commit_message>
Adicionando base padrão SNLP
</commit_message>
<xml_diff>
--- a/bases padrão + cred.xlsx
+++ b/bases padrão + cred.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://myfedex-my.sharepoint.com/personal/guilherme_conceicao_fedex_com/Documents/Documentos/Projetos/Solicitações_SCCT/Welton/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0623004D-D123-4D9B-8492-05778DA04F7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{0623004D-D123-4D9B-8492-05778DA04F7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD079266-0A45-46BD-9969-9D47FA775938}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ABBF3693-6538-4C67-B32B-7AD8D89ACD3B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="217">
   <si>
     <t>BASE_PADRÃO</t>
   </si>
@@ -687,6 +687,9 @@
   </si>
   <si>
     <t>MG FEDEX POLO TEOFILO OTONI</t>
+  </si>
+  <si>
+    <t>Base São Lourenço</t>
   </si>
 </sst>
 </file>
@@ -730,7 +733,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -744,6 +747,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1046,7 +1050,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D791361E-D628-45AA-85DC-89B200D262DC}">
-  <dimension ref="A1:J150"/>
+  <dimension ref="A1:J151"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -2367,6 +2371,14 @@
         <v>215</v>
       </c>
     </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A151" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="B151" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>